<commit_message>
Corrida | GLO-BARL | 2026-03-19 12:06:38.275323
</commit_message>
<xml_diff>
--- a/indicadores/GLO-BARL_out.xlsx
+++ b/indicadores/GLO-BARL_out.xlsx
@@ -107,13 +107,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">11/03/2026</t>
+    <t xml:space="preserve">19/03/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">pcohan</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>

</xml_diff>

<commit_message>
Corrida | GLO-BARL | 2026-06-17 11:28:48.400927
</commit_message>
<xml_diff>
--- a/indicadores/GLO-BARL_out.xlsx
+++ b/indicadores/GLO-BARL_out.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="560">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="562" uniqueCount="562">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -74,6 +74,12 @@
     <t xml:space="preserve">const</t>
   </si>
   <si>
+    <t xml:space="preserve">Alcance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mundo</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resumen del correlograma</t>
   </si>
   <si>
@@ -107,13 +113,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">11/06/2026</t>
+    <t xml:space="preserve">17/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">ysonder</t>
+    <t xml:space="preserve">pcohan</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -2196,9 +2202,13 @@
       <c r="J6" s="1"/>
     </row>
     <row r="7">
-      <c r="A7"/>
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
       <c r="B7"/>
-      <c r="C7"/>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7"/>
@@ -2209,7 +2219,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B8"/>
       <c r="C8"/>
@@ -2223,7 +2233,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B9"/>
       <c r="C9"/>
@@ -2239,7 +2249,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B10"/>
       <c r="C10"/>
@@ -2267,7 +2277,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B12"/>
       <c r="C12"/>
@@ -2281,7 +2291,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B13"/>
       <c r="C13"/>
@@ -2309,7 +2319,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B15"/>
       <c r="C15"/>
@@ -2323,7 +2333,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B16"/>
       <c r="C16"/>
@@ -2337,7 +2347,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -2351,7 +2361,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B18"/>
       <c r="C18"/>
@@ -2367,7 +2377,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B19"/>
       <c r="C19"/>
@@ -2381,7 +2391,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B20"/>
       <c r="C20"/>
@@ -2529,10 +2539,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C32"/>
       <c r="D32"/>
@@ -2545,10 +2555,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B33" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C33"/>
       <c r="D33"/>
@@ -2572,66 +2582,66 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="I1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="K1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="M1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="N1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="O1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="P1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="Q1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="R1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="S1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>97.9979841947098</v>
@@ -2684,7 +2694,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>99.9123235824405</v>
@@ -2741,7 +2751,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>101.256462632428</v>
@@ -2798,7 +2808,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>104.617796969388</v>
@@ -2855,7 +2865,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>102.91405036347</v>
@@ -2912,7 +2922,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>102.211376222997</v>
@@ -2969,7 +2979,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>100.662381741013</v>
@@ -3026,7 +3036,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>96.2405593932116</v>
@@ -3083,7 +3093,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>96.5831222199711</v>
@@ -3140,7 +3150,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>94.242664629166</v>
@@ -3197,7 +3207,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>95.2703436890503</v>
@@ -3254,7 +3264,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>95.3192267086001</v>
@@ -3311,7 +3321,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>97.7613456105595</v>
@@ -3370,7 +3380,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>101.687162246533</v>
@@ -3429,7 +3439,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>102.543981855326</v>
@@ -3488,7 +3498,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>101.731231325723</v>
@@ -3547,7 +3557,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>102.973482706715</v>
@@ -3606,7 +3616,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>105.924732271355</v>
@@ -3665,7 +3675,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>103.509788962501</v>
@@ -3724,7 +3734,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>105.475949864843</v>
@@ -3783,7 +3793,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>105.070436016268</v>
@@ -3842,7 +3852,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>107.224956802485</v>
@@ -3901,7 +3911,7 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>108.502623004872</v>
@@ -3960,7 +3970,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>108.597538621102</v>
@@ -4019,7 +4029,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>107.548745396201</v>
@@ -4078,7 +4088,7 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>104.94110040793</v>
@@ -4137,7 +4147,7 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>106.816045820919</v>
@@ -4196,7 +4206,7 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>104.881361550227</v>
@@ -4255,7 +4265,7 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>104.841975629321</v>
@@ -4314,7 +4324,7 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>106.510347589854</v>
@@ -4373,7 +4383,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>106.390310535065</v>
@@ -4432,7 +4442,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>105.94767419649</v>
@@ -4491,7 +4501,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>108.165600556599</v>
@@ -4550,7 +4560,7 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>107.108112528639</v>
@@ -4609,7 +4619,7 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>110.146131756015</v>
@@ -4668,7 +4678,7 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B37" s="2" t="n">
         <v>108.694911172302</v>
@@ -4727,7 +4737,7 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B38" s="2" t="n">
         <v>108.331958664331</v>
@@ -4786,7 +4796,7 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B39" s="2" t="n">
         <v>106.396795568888</v>
@@ -4845,7 +4855,7 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B40" s="2" t="n">
         <v>102.656155341455</v>
@@ -4904,7 +4914,7 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B41" s="2" t="n">
         <v>102.742428009068</v>
@@ -4963,7 +4973,7 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B42" s="2" t="n">
         <v>101.961133292779</v>
@@ -5022,7 +5032,7 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B43" s="2" t="n">
         <v>98.8051786969787</v>
@@ -5081,7 +5091,7 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B44" s="2" t="n">
         <v>97.5841823822158</v>
@@ -5140,7 +5150,7 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B45" s="2" t="n">
         <v>96.4300044684659</v>
@@ -5199,7 +5209,7 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B46" s="2" t="n">
         <v>95.9936477196356</v>
@@ -5258,7 +5268,7 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B47" s="2" t="n">
         <v>95.523771830646</v>
@@ -5317,7 +5327,7 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B48" s="2" t="n">
         <v>91.0007277495226</v>
@@ -5376,7 +5386,7 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B49" s="2" t="n">
         <v>92.4338524266849</v>
@@ -5435,7 +5445,7 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B50" s="2" t="n">
         <v>92.5392888909269</v>
@@ -5494,7 +5504,7 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B51" s="2" t="n">
         <v>92.6334448028612</v>
@@ -5553,7 +5563,7 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B52" s="2" t="n">
         <v>95.5910590395691</v>
@@ -5612,7 +5622,7 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B53" s="2" t="n">
         <v>94.4281646839013</v>
@@ -5671,7 +5681,7 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B54" s="2" t="n">
         <v>94.3153317269514</v>
@@ -5730,7 +5740,7 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B55" s="2" t="n">
         <v>96.7993602220935</v>
@@ -5789,7 +5799,7 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B56" s="2" t="n">
         <v>100.450072379418</v>
@@ -5848,7 +5858,7 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B57" s="2" t="n">
         <v>101.488119114721</v>
@@ -5907,7 +5917,7 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B58" s="2" t="n">
         <v>100.780548913779</v>
@@ -5966,7 +5976,7 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B59" s="2" t="n">
         <v>100.450934124991</v>
@@ -6025,7 +6035,7 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B60" s="2" t="n">
         <v>101.352609321113</v>
@@ -6084,7 +6094,7 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B61" s="2" t="n">
         <v>100.471426408486</v>
@@ -6143,7 +6153,7 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B62" s="2" t="n">
         <v>99.1679515579239</v>
@@ -6202,7 +6212,7 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B63" s="2" t="n">
         <v>100.681700698621</v>
@@ -6261,7 +6271,7 @@
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B64" s="2" t="n">
         <v>100.202729169027</v>
@@ -6320,7 +6330,7 @@
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B65" s="2" t="n">
         <v>100.843434785948</v>
@@ -6379,7 +6389,7 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B66" s="2" t="n">
         <v>99.9256769203728</v>
@@ -6438,7 +6448,7 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B67" s="2" t="n">
         <v>98.4959429955153</v>
@@ -6497,7 +6507,7 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B68" s="2" t="n">
         <v>96.7731185139848</v>
@@ -6556,7 +6566,7 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B69" s="2" t="n">
         <v>99.2267819586372</v>
@@ -6615,7 +6625,7 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B70" s="2" t="n">
         <v>101.450278095926</v>
@@ -6674,7 +6684,7 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B71" s="2" t="n">
         <v>103.505246984649</v>
@@ -6733,7 +6743,7 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B72" s="2" t="n">
         <v>102.567717629301</v>
@@ -6792,7 +6802,7 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B73" s="2" t="n">
         <v>100.624299434717</v>
@@ -6851,7 +6861,7 @@
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B74" s="2" t="n">
         <v>97.9120823689786</v>
@@ -6910,7 +6920,7 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B75" s="2" t="n">
         <v>96.4036834696806</v>
@@ -6969,7 +6979,7 @@
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B76" s="2" t="n">
         <v>95.0188760349786</v>
@@ -7028,7 +7038,7 @@
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B77" s="2" t="n">
         <v>94.0853417974893</v>
@@ -7087,7 +7097,7 @@
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B78" s="2" t="n">
         <v>93.702561010835</v>
@@ -7146,7 +7156,7 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B79" s="2" t="n">
         <v>94.0333035219863</v>
@@ -7205,7 +7215,7 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B80" s="2" t="n">
         <v>94.2140450195869</v>
@@ -7264,7 +7274,7 @@
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B81" s="2" t="n">
         <v>92.253125612917</v>
@@ -7323,7 +7333,7 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B82" s="2" t="n">
         <v>90.8121704679221</v>
@@ -7382,7 +7392,7 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B83" s="2" t="n">
         <v>87.8543542743344</v>
@@ -7441,7 +7451,7 @@
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B84" s="2" t="n">
         <v>88.6226483913793</v>
@@ -7500,7 +7510,7 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B85" s="2" t="n">
         <v>90.428716847154</v>
@@ -7559,7 +7569,7 @@
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B86" s="2" t="n">
         <v>94.1907862868507</v>
@@ -7618,7 +7628,7 @@
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B87" s="2" t="n">
         <v>95.6907330161598</v>
@@ -7677,7 +7687,7 @@
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B88" s="2" t="n">
         <v>97.0536213380009</v>
@@ -7736,7 +7746,7 @@
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B89" s="2" t="n">
         <v>99.3134193333442</v>
@@ -7795,7 +7805,7 @@
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B90" s="2" t="n">
         <v>105.251318732609</v>
@@ -7854,7 +7864,7 @@
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B91" s="2" t="n">
         <v>108.853199921229</v>
@@ -7913,7 +7923,7 @@
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B92" s="2" t="n">
         <v>115.610624250758</v>
@@ -7972,7 +7982,7 @@
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B93" s="2" t="n">
         <v>109.383641521983</v>
@@ -8031,7 +8041,7 @@
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B94" s="2" t="n">
         <v>107.390523190467</v>
@@ -8090,7 +8100,7 @@
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B95" s="2" t="n">
         <v>106.96336679399</v>
@@ -8149,7 +8159,7 @@
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B96" s="2" t="n">
         <v>109.902660029799</v>
@@ -8208,7 +8218,7 @@
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B97" s="2" t="n">
         <v>108.642077225997</v>
@@ -8267,7 +8277,7 @@
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B98" s="2" t="n">
         <v>110.197907375524</v>
@@ -8326,7 +8336,7 @@
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B99" s="2" t="n">
         <v>115.410700774384</v>
@@ -8385,7 +8395,7 @@
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B100" s="2" t="n">
         <v>109.666759747917</v>
@@ -8444,7 +8454,7 @@
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B101" s="2" t="n">
         <v>116.766029584194</v>
@@ -8503,7 +8513,7 @@
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B102" s="2" t="n">
         <v>116.028592692965</v>
@@ -8562,7 +8572,7 @@
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B103" s="2" t="n">
         <v>106.579572751446</v>
@@ -8621,7 +8631,7 @@
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B104" s="2" t="n">
         <v>101.293090694213</v>
@@ -8680,7 +8690,7 @@
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B105" s="2" t="n">
         <v>102.956817139608</v>
@@ -8739,7 +8749,7 @@
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B106" s="2" t="n">
         <v>99.4674866350279</v>
@@ -8798,7 +8808,7 @@
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B107" s="2" t="n">
         <v>99.1357191079965</v>
@@ -8857,7 +8867,7 @@
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B108" s="2" t="n">
         <v>98.4303317047678</v>
@@ -8916,7 +8926,7 @@
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B109" s="2" t="n">
         <v>97.4156761485321</v>
@@ -8975,7 +8985,7 @@
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B110" s="2" t="n">
         <v>93.9629575386618</v>
@@ -9034,7 +9044,7 @@
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B111" s="2" t="n">
         <v>88.9234458381353</v>
@@ -9093,7 +9103,7 @@
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B112" s="2" t="n">
         <v>87.5459571693465</v>
@@ -9152,7 +9162,7 @@
     </row>
     <row r="113">
       <c r="A113" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B113" s="2" t="n">
         <v>80.0433437491058</v>
@@ -9211,7 +9221,7 @@
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B114" s="2" t="n">
         <v>80.1755884851704</v>
@@ -9270,7 +9280,7 @@
     </row>
     <row r="115">
       <c r="A115" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B115" s="2" t="n">
         <v>83.7459954448804</v>
@@ -9329,7 +9339,7 @@
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B116" s="2" t="n">
         <v>84.5553351804783</v>
@@ -9388,7 +9398,7 @@
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B117" s="2" t="n">
         <v>83.1296653535657</v>
@@ -9447,7 +9457,7 @@
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B118" s="2" t="n">
         <v>85.8675931682814</v>
@@ -9506,7 +9516,7 @@
     </row>
     <row r="119">
       <c r="A119" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B119" s="2" t="n">
         <v>81.2720526032554</v>
@@ -9565,7 +9575,7 @@
     </row>
     <row r="120">
       <c r="A120" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B120" s="2" t="n">
         <v>78.3852092325461</v>
@@ -9624,7 +9634,7 @@
     </row>
     <row r="121">
       <c r="A121" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B121" s="2" t="n">
         <v>78.2015108999537</v>
@@ -9683,7 +9693,7 @@
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B122" s="2" t="n">
         <v>89.8332805731024</v>
@@ -9742,7 +9752,7 @@
     </row>
     <row r="123">
       <c r="A123" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B123" s="2" t="n">
         <v>92.2679090079602</v>
@@ -9801,7 +9811,7 @@
     </row>
     <row r="124">
       <c r="A124" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B124" s="2" t="n">
         <v>100.20271463093</v>
@@ -9860,7 +9870,7 @@
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B125" s="2" t="n">
         <v>106.392046068454</v>
@@ -9919,7 +9929,7 @@
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B126" s="2" t="n">
         <v>112.735140608008</v>
@@ -9978,7 +9988,7 @@
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B127" s="2" t="n">
         <v>111.798612300267</v>
@@ -10037,7 +10047,7 @@
     </row>
     <row r="128">
       <c r="A128" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B128" s="2" t="n">
         <v>110.379927985984</v>
@@ -10096,7 +10106,7 @@
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B129" s="2" t="n">
         <v>108.590268520063</v>
@@ -10155,7 +10165,7 @@
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B130" s="2" t="n">
         <v>104.500281281591</v>
@@ -10214,7 +10224,7 @@
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B131" s="2" t="n">
         <v>106.424839296461</v>
@@ -10273,7 +10283,7 @@
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B132" s="2" t="n">
         <v>107.241259307763</v>
@@ -10332,7 +10342,7 @@
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B133" s="2" t="n">
         <v>109.651271614475</v>
@@ -10391,7 +10401,7 @@
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B134" s="2" t="n">
         <v>104.540698297143</v>
@@ -10450,7 +10460,7 @@
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B135" s="2" t="n">
         <v>103.818333613893</v>
@@ -10509,7 +10519,7 @@
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B136" s="2" t="n">
         <v>102.867757112229</v>
@@ -10568,7 +10578,7 @@
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B137" s="2" t="n">
         <v>98.482624307665</v>
@@ -10627,7 +10637,7 @@
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B138" s="2" t="n">
         <v>92.7553077312099</v>
@@ -10686,7 +10696,7 @@
     </row>
     <row r="139">
       <c r="A139" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B139" s="2" t="n">
         <v>93.727368357635</v>
@@ -10745,7 +10755,7 @@
     </row>
     <row r="140">
       <c r="A140" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B140" s="2" t="n">
         <v>96.6766320193648</v>
@@ -10804,7 +10814,7 @@
     </row>
     <row r="141">
       <c r="A141" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B141" s="2" t="n">
         <v>98.7565551244898</v>
@@ -10863,7 +10873,7 @@
     </row>
     <row r="142">
       <c r="A142" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B142" s="2" t="n">
         <v>104.433157982442</v>
@@ -10922,7 +10932,7 @@
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B143" s="2" t="n">
         <v>106.630180545243</v>
@@ -10981,7 +10991,7 @@
     </row>
     <row r="144">
       <c r="A144" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B144" s="2" t="n">
         <v>111.96224814386</v>
@@ -11040,7 +11050,7 @@
     </row>
     <row r="145">
       <c r="A145" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B145" s="2" t="n">
         <v>110.618969680857</v>
@@ -11099,7 +11109,7 @@
     </row>
     <row r="146">
       <c r="A146" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B146" s="2" t="n">
         <v>111.993038692346</v>
@@ -11158,7 +11168,7 @@
     </row>
     <row r="147">
       <c r="A147" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B147" s="2" t="n">
         <v>107.522295133376</v>
@@ -11217,7 +11227,7 @@
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B148" s="2" t="n">
         <v>108.30981667245</v>
@@ -11276,7 +11286,7 @@
     </row>
     <row r="149">
       <c r="A149" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B149" s="2" t="n">
         <v>110.643406922888</v>
@@ -11335,7 +11345,7 @@
     </row>
     <row r="150">
       <c r="A150" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B150" s="2" t="n">
         <v>114.939120919706</v>
@@ -11394,7 +11404,7 @@
     </row>
     <row r="151">
       <c r="A151" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B151" s="2" t="n">
         <v>116.031915227963</v>
@@ -11453,7 +11463,7 @@
     </row>
     <row r="152">
       <c r="A152" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B152" s="2" t="n">
         <v>115.136581114543</v>
@@ -11512,7 +11522,7 @@
     </row>
     <row r="153">
       <c r="A153" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B153" s="2" t="n">
         <v>109.355584200007</v>
@@ -11571,7 +11581,7 @@
     </row>
     <row r="154">
       <c r="A154" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B154" s="2" t="n">
         <v>107.921836729549</v>
@@ -11630,7 +11640,7 @@
     </row>
     <row r="155">
       <c r="A155" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B155" s="2" t="n">
         <v>106.041586581965</v>
@@ -11689,7 +11699,7 @@
     </row>
     <row r="156">
       <c r="A156" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B156" s="2" t="n">
         <v>101.260337277202</v>
@@ -11748,7 +11758,7 @@
     </row>
     <row r="157">
       <c r="A157" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B157" s="2" t="n">
         <v>100.454177074741</v>
@@ -11807,7 +11817,7 @@
     </row>
     <row r="158">
       <c r="A158" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B158" s="2" t="n">
         <v>99.1827846946181</v>
@@ -11866,7 +11876,7 @@
     </row>
     <row r="159">
       <c r="A159" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B159" s="2" t="n">
         <v>106.075001170341</v>
@@ -11925,7 +11935,7 @@
     </row>
     <row r="160">
       <c r="A160" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B160" s="2" t="n">
         <v>107.279998513938</v>
@@ -11984,7 +11994,7 @@
     </row>
     <row r="161">
       <c r="A161" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B161" s="2" t="n">
         <v>104.403014899349</v>
@@ -12043,7 +12053,7 @@
     </row>
     <row r="162">
       <c r="A162" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B162" s="2" t="n">
         <v>98.7222967721598</v>
@@ -12102,7 +12112,7 @@
     </row>
     <row r="163">
       <c r="A163" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B163" s="2" t="n">
         <v>97.9101338167646</v>
@@ -12161,7 +12171,7 @@
     </row>
     <row r="164">
       <c r="A164" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B164" s="2" t="n">
         <v>97.2923841958559</v>
@@ -12220,7 +12230,7 @@
     </row>
     <row r="165">
       <c r="A165" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B165" s="2" t="n">
         <v>99.839146643182</v>
@@ -12279,7 +12289,7 @@
     </row>
     <row r="166">
       <c r="A166" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B166" s="2" t="n">
         <v>100.835577949218</v>
@@ -12338,7 +12348,7 @@
     </row>
     <row r="167">
       <c r="A167" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B167" s="2" t="n">
         <v>102.158657474214</v>
@@ -12397,7 +12407,7 @@
     </row>
     <row r="168">
       <c r="A168" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B168" s="2" t="n">
         <v>102.661073861553</v>
@@ -12456,7 +12466,7 @@
     </row>
     <row r="169">
       <c r="A169" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B169" s="2" t="n">
         <v>104.338861401024</v>
@@ -12515,7 +12525,7 @@
     </row>
     <row r="170">
       <c r="A170" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B170" s="2" t="n">
         <v>104.580977957206</v>
@@ -12574,7 +12584,7 @@
     </row>
     <row r="171">
       <c r="A171" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B171" s="2" t="n">
         <v>105.651955087103</v>
@@ -12633,7 +12643,7 @@
     </row>
     <row r="172">
       <c r="A172" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B172" s="2" t="n">
         <v>104.853026520402</v>
@@ -12692,7 +12702,7 @@
     </row>
     <row r="173">
       <c r="A173" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B173" s="2" t="n">
         <v>106.025349357157</v>
@@ -12751,7 +12761,7 @@
     </row>
     <row r="174">
       <c r="A174" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B174" s="2" t="n">
         <v>107.330348118735</v>
@@ -12810,7 +12820,7 @@
     </row>
     <row r="175">
       <c r="A175" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B175" s="2" t="n">
         <v>108.574900044069</v>
@@ -12869,7 +12879,7 @@
     </row>
     <row r="176">
       <c r="A176" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B176" s="2" t="n">
         <v>107.949930683617</v>
@@ -12928,7 +12938,7 @@
     </row>
     <row r="177">
       <c r="A177" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B177" s="2" t="n">
         <v>105.234815227485</v>
@@ -12987,7 +12997,7 @@
     </row>
     <row r="178">
       <c r="A178" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B178" s="2" t="n">
         <v>104.996495686912</v>
@@ -13046,7 +13056,7 @@
     </row>
     <row r="179">
       <c r="A179" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B179" s="2" t="n">
         <v>106.111271273005</v>
@@ -13105,7 +13115,7 @@
     </row>
     <row r="180">
       <c r="A180" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B180" s="2" t="n">
         <v>108.141933052115</v>
@@ -13164,7 +13174,7 @@
     </row>
     <row r="181">
       <c r="A181" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B181" s="2" t="n">
         <v>109.241010123342</v>
@@ -13223,7 +13233,7 @@
     </row>
     <row r="182">
       <c r="A182" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B182" s="2" t="n">
         <v>109.369588423845</v>
@@ -13282,7 +13292,7 @@
     </row>
     <row r="183">
       <c r="A183" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B183" s="2" t="n">
         <v>108.910630291483</v>
@@ -13341,7 +13351,7 @@
     </row>
     <row r="184">
       <c r="A184" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B184" s="2" t="n">
         <v>108.242535483088</v>
@@ -13400,7 +13410,7 @@
     </row>
     <row r="185">
       <c r="A185" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B185" s="2" t="n">
         <v>108.38229350618</v>
@@ -13459,7 +13469,7 @@
     </row>
     <row r="186">
       <c r="A186" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B186" s="2" t="n">
         <v>105.080777221884</v>
@@ -13518,7 +13528,7 @@
     </row>
     <row r="187">
       <c r="A187" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B187" s="2" t="n">
         <v>102.727189262837</v>
@@ -13577,7 +13587,7 @@
     </row>
     <row r="188">
       <c r="A188" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B188" s="2" t="n">
         <v>104.498959189735</v>
@@ -13636,7 +13646,7 @@
     </row>
     <row r="189">
       <c r="A189" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B189" s="2" t="n">
         <v>104.802565687022</v>
@@ -13695,7 +13705,7 @@
     </row>
     <row r="190">
       <c r="A190" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B190" s="2" t="n">
         <v>105.536883363506</v>
@@ -13754,7 +13764,7 @@
     </row>
     <row r="191">
       <c r="A191" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B191" s="2" t="n">
         <v>104.776055990604</v>
@@ -13813,7 +13823,7 @@
     </row>
     <row r="192">
       <c r="A192" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B192" s="2" t="n">
         <v>102.523606311132</v>
@@ -13872,7 +13882,7 @@
     </row>
     <row r="193">
       <c r="A193" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B193" s="2" t="n">
         <v>104.01034831381</v>
@@ -13931,7 +13941,7 @@
     </row>
     <row r="194">
       <c r="A194" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B194" s="2" t="n">
         <v>102.89602073993</v>
@@ -13990,7 +14000,7 @@
     </row>
     <row r="195">
       <c r="A195" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B195" s="2" t="n">
         <v>99.4622469583722</v>
@@ -14049,7 +14059,7 @@
     </row>
     <row r="196">
       <c r="A196" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B196" s="2" t="n">
         <v>98.6645734455728</v>
@@ -14108,7 +14118,7 @@
     </row>
     <row r="197">
       <c r="A197" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B197" s="2" t="n">
         <v>97.2834029612259</v>
@@ -14167,7 +14177,7 @@
     </row>
     <row r="198">
       <c r="A198" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B198" s="2" t="n">
         <v>93.5174253261584</v>
@@ -14226,7 +14236,7 @@
     </row>
     <row r="199">
       <c r="A199" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B199" s="2" t="n">
         <v>91.6249702330932</v>
@@ -14285,7 +14295,7 @@
     </row>
     <row r="200">
       <c r="A200" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B200" s="2" t="n">
         <v>89.4730626241167</v>
@@ -14344,7 +14354,7 @@
     </row>
     <row r="201">
       <c r="A201" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B201" s="2" t="n">
         <v>87.3804753281206</v>
@@ -14403,7 +14413,7 @@
     </row>
     <row r="202">
       <c r="A202" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B202" s="2" t="n">
         <v>86.8026357329618</v>
@@ -14462,7 +14472,7 @@
     </row>
     <row r="203">
       <c r="A203" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B203" s="2" t="n">
         <v>83.5789078831221</v>
@@ -14521,7 +14531,7 @@
     </row>
     <row r="204">
       <c r="A204" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B204" s="2" t="n">
         <v>69.1951803888895</v>
@@ -14580,7 +14590,7 @@
     </row>
     <row r="205">
       <c r="A205" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B205" s="2" t="n">
         <v>56.1900096921658</v>
@@ -14639,7 +14649,7 @@
     </row>
     <row r="206">
       <c r="A206" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B206" s="2" t="n">
         <v>53.4656594551293</v>
@@ -14698,7 +14708,7 @@
     </row>
     <row r="207">
       <c r="A207" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B207" s="2" t="n">
         <v>57.1183989178281</v>
@@ -14757,7 +14767,7 @@
     </row>
     <row r="208">
       <c r="A208" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B208" s="2" t="n">
         <v>63.0649399206152</v>
@@ -14816,7 +14826,7 @@
     </row>
     <row r="209">
       <c r="A209" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B209" s="2" t="n">
         <v>65.882357797124</v>
@@ -14875,7 +14885,7 @@
     </row>
     <row r="210">
       <c r="A210" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B210" s="2" t="n">
         <v>80.2257392454932</v>
@@ -14934,7 +14944,7 @@
     </row>
     <row r="211">
       <c r="A211" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B211" s="2" t="n">
         <v>86.5282033214669</v>
@@ -14993,7 +15003,7 @@
     </row>
     <row r="212">
       <c r="A212" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B212" s="2" t="n">
         <v>93.4252537623751</v>
@@ -15052,7 +15062,7 @@
     </row>
     <row r="213">
       <c r="A213" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B213" s="2" t="n">
         <v>98.522970826149</v>
@@ -15111,7 +15121,7 @@
     </row>
     <row r="214">
       <c r="A214" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B214" s="2" t="n">
         <v>103.022996295824</v>
@@ -15170,7 +15180,7 @@
     </row>
     <row r="215">
       <c r="A215" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B215" s="2" t="n">
         <v>103.92773558546</v>
@@ -15229,7 +15239,7 @@
     </row>
     <row r="216">
       <c r="A216" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B216" s="2" t="n">
         <v>114.038313760854</v>
@@ -15288,7 +15298,7 @@
     </row>
     <row r="217">
       <c r="A217" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B217" s="2" t="n">
         <v>115.973686567686</v>
@@ -15347,7 +15357,7 @@
     </row>
     <row r="218">
       <c r="A218" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B218" s="2" t="n">
         <v>121.232774581114</v>
@@ -15406,7 +15416,7 @@
     </row>
     <row r="219">
       <c r="A219" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B219" s="2" t="n">
         <v>123.789679520558</v>
@@ -15465,7 +15475,7 @@
     </row>
     <row r="220">
       <c r="A220" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B220" s="2" t="n">
         <v>121.369167010795</v>
@@ -15524,7 +15534,7 @@
     </row>
     <row r="221">
       <c r="A221" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B221" s="2" t="n">
         <v>124.22570986689</v>
@@ -15583,7 +15593,7 @@
     </row>
     <row r="222">
       <c r="A222" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B222" s="2" t="n">
         <v>122.039547616672</v>
@@ -15642,7 +15652,7 @@
     </row>
     <row r="223">
       <c r="A223" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B223" s="2" t="n">
         <v>121.496758965121</v>
@@ -15701,7 +15711,7 @@
     </row>
     <row r="224">
       <c r="A224" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B224" s="2" t="n">
         <v>115.105210578609</v>
@@ -15760,7 +15770,7 @@
     </row>
     <row r="225">
       <c r="A225" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B225" s="2" t="n">
         <v>112.017740804911</v>
@@ -15819,7 +15829,7 @@
     </row>
     <row r="226">
       <c r="A226" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B226" s="2" t="n">
         <v>107.775840371295</v>
@@ -15878,7 +15888,7 @@
     </row>
     <row r="227">
       <c r="A227" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B227" s="2" t="n">
         <v>109.847402979905</v>
@@ -15937,7 +15947,7 @@
     </row>
     <row r="228">
       <c r="A228" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B228" s="2" t="n">
         <v>108.558511414794</v>
@@ -15996,7 +16006,7 @@
     </row>
     <row r="229">
       <c r="A229" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B229" s="2" t="n">
         <v>111.770399818639</v>
@@ -16055,7 +16065,7 @@
     </row>
     <row r="230">
       <c r="A230" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B230" s="2" t="n">
         <v>109.647299950891</v>
@@ -16114,7 +16124,7 @@
     </row>
     <row r="231">
       <c r="A231" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B231" s="2" t="n">
         <v>107.806915480704</v>
@@ -16173,7 +16183,7 @@
     </row>
     <row r="232">
       <c r="A232" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B232" s="2" t="n">
         <v>109.061149684447</v>
@@ -16232,7 +16242,7 @@
     </row>
     <row r="233">
       <c r="A233" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B233" s="2" t="n">
         <v>104.276303603806</v>
@@ -16291,7 +16301,7 @@
     </row>
     <row r="234">
       <c r="A234" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B234" s="2" t="n">
         <v>97.2713426302843</v>
@@ -16350,7 +16360,7 @@
     </row>
     <row r="235">
       <c r="A235" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B235" s="2" t="n">
         <v>98.836813398166</v>
@@ -16409,7 +16419,7 @@
     </row>
     <row r="236">
       <c r="A236" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B236" s="2" t="n">
         <v>99.2870355949033</v>
@@ -16468,7 +16478,7 @@
     </row>
     <row r="237">
       <c r="A237" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B237" s="2" t="n">
         <v>102.185109370432</v>
@@ -16527,7 +16537,7 @@
     </row>
     <row r="238">
       <c r="A238" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B238" s="2" t="n">
         <v>101.513108436034</v>
@@ -16586,7 +16596,7 @@
     </row>
     <row r="239">
       <c r="A239" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B239" s="2" t="n">
         <v>98.7478789828572</v>
@@ -16645,7 +16655,7 @@
     </row>
     <row r="240">
       <c r="A240" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B240" s="2" t="n">
         <v>95.5672703123822</v>
@@ -16704,7 +16714,7 @@
     </row>
     <row r="241">
       <c r="A241" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B241" s="2" t="n">
         <v>93.2119466352712</v>
@@ -16763,7 +16773,7 @@
     </row>
     <row r="242">
       <c r="A242" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B242" s="2" t="n">
         <v>93.4349865695764</v>
@@ -16822,7 +16832,7 @@
     </row>
     <row r="243">
       <c r="A243" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B243" s="2" t="n">
         <v>92.885616746522</v>
@@ -16881,7 +16891,7 @@
     </row>
     <row r="244">
       <c r="A244" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B244" s="2" t="n">
         <v>95.4461147411491</v>
@@ -16940,7 +16950,7 @@
     </row>
     <row r="245">
       <c r="A245" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B245" s="2" t="n">
         <v>96.2051824386935</v>
@@ -16999,7 +17009,7 @@
     </row>
     <row r="246">
       <c r="A246" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="B246" s="2" t="n">
         <v>97.0247286682173</v>
@@ -17058,7 +17068,7 @@
     </row>
     <row r="247">
       <c r="A247" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B247" s="2" t="n">
         <v>92.7729711513459</v>
@@ -17117,7 +17127,7 @@
     </row>
     <row r="248">
       <c r="A248" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B248" s="2" t="n">
         <v>91.6937869269612</v>
@@ -17176,7 +17186,7 @@
     </row>
     <row r="249">
       <c r="A249" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B249" s="2" t="n">
         <v>91.4595456218406</v>
@@ -17235,7 +17245,7 @@
     </row>
     <row r="250">
       <c r="A250" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B250" s="2" t="n">
         <v>91.4474902219512</v>
@@ -17294,7 +17304,7 @@
     </row>
     <row r="251">
       <c r="A251" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B251" s="2" t="n">
         <v>92.3544476504463</v>
@@ -17353,7 +17363,7 @@
     </row>
     <row r="252">
       <c r="A252" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B252" s="2" t="n">
         <v>91.9787063230802</v>
@@ -17412,7 +17422,7 @@
     </row>
     <row r="253">
       <c r="A253" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B253" s="2" t="n">
         <v>94.2326075606328</v>
@@ -17471,7 +17481,7 @@
     </row>
     <row r="254">
       <c r="A254" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B254" s="2" t="n">
         <v>97.098549103585</v>
@@ -17530,7 +17540,7 @@
     </row>
     <row r="255">
       <c r="A255" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B255" s="2" t="n">
         <v>102.737042717651</v>
@@ -17589,7 +17599,7 @@
     </row>
     <row r="256">
       <c r="A256" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B256" s="2" t="n">
         <v>102.667138857139</v>
@@ -17648,7 +17658,7 @@
     </row>
     <row r="257">
       <c r="A257" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B257" s="2" t="n">
         <v>104.190552860144</v>
@@ -17707,7 +17717,7 @@
     </row>
     <row r="258">
       <c r="A258" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B258" s="2" t="n">
         <v>100.871334246041</v>
@@ -17766,7 +17776,7 @@
     </row>
     <row r="259">
       <c r="A259" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B259" s="2" t="n">
         <v>103.064737915418</v>
@@ -17825,7 +17835,7 @@
     </row>
     <row r="260">
       <c r="A260" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B260" s="2" t="n">
         <v>105.689064465603</v>
@@ -17884,7 +17894,7 @@
     </row>
     <row r="261">
       <c r="A261" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B261" s="2" t="n">
         <v>105.442275546092</v>
@@ -17943,7 +17953,7 @@
     </row>
     <row r="262">
       <c r="A262" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B262" s="2" t="n">
         <v>108.165860110382</v>
@@ -18002,7 +18012,7 @@
     </row>
     <row r="263">
       <c r="A263" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B263" s="2" t="n">
         <v>108.443437705929</v>
@@ -18061,7 +18071,7 @@
     </row>
     <row r="264">
       <c r="A264" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B264" s="2" t="n">
         <v>109.862803844108</v>
@@ -18120,7 +18130,7 @@
     </row>
     <row r="265">
       <c r="A265" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B265" s="2" t="n">
         <v>109.662948595782</v>
@@ -18179,7 +18189,7 @@
     </row>
     <row r="266">
       <c r="A266" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B266" s="2" t="n">
         <v>108.016726536003</v>
@@ -18238,7 +18248,7 @@
     </row>
     <row r="267">
       <c r="A267" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B267" s="2" t="n">
         <v>106.746379679847</v>
@@ -18297,7 +18307,7 @@
     </row>
     <row r="268">
       <c r="A268" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B268" s="2" t="n">
         <v>105.912179488779</v>
@@ -18356,7 +18366,7 @@
     </row>
     <row r="269">
       <c r="A269" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B269" s="2" t="n">
         <v>102.146065909443</v>
@@ -18415,7 +18425,7 @@
     </row>
     <row r="270">
       <c r="A270" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B270" s="2" t="n">
         <v>103.387834172621</v>
@@ -18474,7 +18484,7 @@
     </row>
     <row r="271">
       <c r="A271" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B271" s="2" t="n">
         <v>103.694783791458</v>
@@ -18533,7 +18543,7 @@
     </row>
     <row r="272">
       <c r="A272" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="B272" s="2" t="n">
         <v>102.87924695396</v>
@@ -18592,7 +18602,7 @@
     </row>
     <row r="273">
       <c r="A273" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B273" s="2" t="n">
         <v>104.819018494828</v>
@@ -18651,7 +18661,7 @@
     </row>
     <row r="274">
       <c r="A274" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B274" s="2" t="n">
         <v>103.009355223058</v>
@@ -18710,7 +18720,7 @@
     </row>
     <row r="275">
       <c r="A275" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B275" s="2" t="n">
         <v>103.065111385226</v>
@@ -18769,7 +18779,7 @@
     </row>
     <row r="276">
       <c r="A276" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B276" s="2" t="n">
         <v>102.435626896494</v>
@@ -18828,7 +18838,7 @@
     </row>
     <row r="277">
       <c r="A277" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B277" s="2" t="n">
         <v>100.538619217064</v>
@@ -18887,7 +18897,7 @@
     </row>
     <row r="278">
       <c r="A278" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B278" s="2" t="n">
         <v>96.9327843194228</v>
@@ -18946,7 +18956,7 @@
     </row>
     <row r="279">
       <c r="A279" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B279" s="2" t="n">
         <v>96.6820748627584</v>
@@ -19005,7 +19015,7 @@
     </row>
     <row r="280">
       <c r="A280" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B280" s="2" t="n">
         <v>95.4641303586889</v>
@@ -19064,7 +19074,7 @@
     </row>
     <row r="281">
       <c r="A281" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B281" s="2" t="n">
         <v>97.2207684782083</v>
@@ -19123,7 +19133,7 @@
     </row>
     <row r="282">
       <c r="A282" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B282" s="2" t="n">
         <v>97.1688089599386</v>
@@ -19182,7 +19192,7 @@
     </row>
     <row r="283">
       <c r="A283" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B283" s="2" t="n">
         <v>96.8960886546879</v>
@@ -19241,7 +19251,7 @@
     </row>
     <row r="284">
       <c r="A284" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B284" s="2" t="n">
         <v>95.0656968534507</v>
@@ -19300,7 +19310,7 @@
     </row>
     <row r="285">
       <c r="A285" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B285" s="2" t="n">
         <v>95.7977923992184</v>
@@ -19359,7 +19369,7 @@
     </row>
     <row r="286">
       <c r="A286" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B286" s="2" t="n">
         <v>93.2587849771851</v>
@@ -19418,7 +19428,7 @@
     </row>
     <row r="287">
       <c r="A287" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B287" s="2" t="n">
         <v>90.8976118905353</v>
@@ -19477,7 +19487,7 @@
     </row>
     <row r="288">
       <c r="A288" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B288" s="2" t="n">
         <v>91.7411689545185</v>
@@ -19536,7 +19546,7 @@
     </row>
     <row r="289">
       <c r="A289" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B289" s="2" t="n">
         <v>93.402734906208</v>
@@ -19595,7 +19605,7 @@
     </row>
     <row r="290">
       <c r="A290" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B290" s="2" t="n">
         <v>95.9460883502636</v>
@@ -19654,7 +19664,7 @@
     </row>
     <row r="291">
       <c r="A291" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B291" s="2" t="n">
         <v>95.5901886228901</v>
@@ -19713,7 +19723,7 @@
     </row>
     <row r="292">
       <c r="A292" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B292" s="2" t="n">
         <v>93.9049643359219</v>
@@ -19772,7 +19782,7 @@
     </row>
     <row r="293">
       <c r="A293" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B293" s="2" t="n">
         <v>96.2268159279917</v>
@@ -19831,7 +19841,7 @@
     </row>
     <row r="294">
       <c r="A294" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="B294" s="2" t="n">
         <v>99.8102874265049</v>
@@ -19890,7 +19900,7 @@
     </row>
     <row r="295">
       <c r="A295" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B295" s="2" t="n">
         <v>100.021766062744</v>
@@ -19949,7 +19959,7 @@
     </row>
     <row r="296">
       <c r="A296" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="B296" s="2" t="n">
         <v>100.887817887854</v>
@@ -20008,7 +20018,7 @@
     </row>
     <row r="297">
       <c r="A297" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B297" s="2" t="n">
         <v>101.809637209826</v>
@@ -20067,7 +20077,7 @@
     </row>
     <row r="298">
       <c r="A298" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B298" s="2" t="n">
         <v>105.122483799231</v>
@@ -20126,7 +20136,7 @@
     </row>
     <row r="299">
       <c r="A299" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B299" s="2" t="n">
         <v>107.39932797971</v>
@@ -20185,7 +20195,7 @@
     </row>
     <row r="300">
       <c r="A300" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B300" s="2" t="n">
         <v>109.038591135776</v>
@@ -20244,7 +20254,7 @@
     </row>
     <row r="301">
       <c r="A301" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B301" s="2" t="n">
         <v>109.938446289945</v>
@@ -20303,7 +20313,7 @@
     </row>
     <row r="302">
       <c r="A302" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B302" s="2" t="n">
         <v>110.56640503568</v>
@@ -20362,7 +20372,7 @@
     </row>
     <row r="303">
       <c r="A303" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B303" s="2" t="n">
         <v>113.180027384931</v>
@@ -20421,7 +20431,7 @@
     </row>
     <row r="304">
       <c r="A304" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B304" s="2" t="n">
         <v>114.571446409031</v>
@@ -20480,7 +20490,7 @@
     </row>
     <row r="305">
       <c r="A305" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B305" s="2" t="n">
         <v>114.759739478556</v>
@@ -20539,7 +20549,7 @@
     </row>
     <row r="306">
       <c r="A306" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B306" s="2" t="n">
         <v>112.487757922968</v>
@@ -20598,7 +20608,7 @@
     </row>
     <row r="307">
       <c r="A307" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B307" s="2" t="n">
         <v>114.087723458378</v>
@@ -20657,7 +20667,7 @@
     </row>
     <row r="308">
       <c r="A308" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B308" s="2" t="n">
         <v>115.090185947961</v>
@@ -20716,7 +20726,7 @@
     </row>
     <row r="309">
       <c r="A309" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B309" s="2" t="n">
         <v>112.681075481269</v>
@@ -20775,7 +20785,7 @@
     </row>
     <row r="310">
       <c r="A310" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B310" s="2" t="n">
         <v>112.377275628373</v>
@@ -20834,7 +20844,7 @@
     </row>
     <row r="311">
       <c r="A311" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B311" s="2" t="n">
         <v>113.433788053568</v>
@@ -20893,7 +20903,7 @@
     </row>
     <row r="312">
       <c r="A312" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="B312" s="2" t="n">
         <v>112.370251517323</v>
@@ -20952,7 +20962,7 @@
     </row>
     <row r="313">
       <c r="A313" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B313" s="2" t="n">
         <v>110.669370521278</v>
@@ -21011,7 +21021,7 @@
     </row>
     <row r="314">
       <c r="A314" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B314" s="2" t="n">
         <v>109.287231672456</v>
@@ -21070,7 +21080,7 @@
     </row>
     <row r="315">
       <c r="A315" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B315" s="2" t="n">
         <v>108.021889440532</v>
@@ -21129,7 +21139,7 @@
     </row>
     <row r="316">
       <c r="A316" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="B316" s="2" t="n">
         <v>105.804317101153</v>
@@ -21188,7 +21198,7 @@
     </row>
     <row r="317">
       <c r="A317" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B317" s="2" t="n">
         <v>104.038668740825</v>
@@ -21247,7 +21257,7 @@
     </row>
     <row r="318">
       <c r="A318" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B318" s="2" t="n">
         <v>102.449995136436</v>
@@ -21306,7 +21316,7 @@
     </row>
     <row r="319">
       <c r="A319" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="B319" s="2" t="n">
         <v>102.719072951972</v>
@@ -21365,7 +21375,7 @@
     </row>
     <row r="320">
       <c r="A320" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="B320" s="2" t="n">
         <v>101.464155646726</v>
@@ -21424,7 +21434,7 @@
     </row>
     <row r="321">
       <c r="A321" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B321" s="2" t="n">
         <v>100.528382207224</v>
@@ -21483,7 +21493,7 @@
     </row>
     <row r="322">
       <c r="A322" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="B322" s="2" t="n">
         <v>97.4559598158932</v>
@@ -21542,7 +21552,7 @@
     </row>
     <row r="323">
       <c r="A323" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B323" s="2" t="n">
         <v>95.1604910870211</v>
@@ -21601,7 +21611,7 @@
     </row>
     <row r="324">
       <c r="A324" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="B324" s="2" t="n">
         <v>94.431371765584</v>
@@ -21660,7 +21670,7 @@
     </row>
     <row r="325">
       <c r="A325" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B325" s="2" t="n">
         <v>93.6529591489364</v>
@@ -21719,7 +21729,7 @@
     </row>
     <row r="326">
       <c r="A326" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="B326" s="2" t="n">
         <v>93.3446383423321</v>
@@ -21778,7 +21788,7 @@
     </row>
     <row r="327">
       <c r="A327" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B327" s="2" t="n">
         <v>90.288508073767</v>
@@ -21837,7 +21847,7 @@
     </row>
     <row r="328">
       <c r="A328" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="B328" s="2" t="n">
         <v>92.1423058746909</v>
@@ -21896,7 +21906,7 @@
     </row>
     <row r="329">
       <c r="A329" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B329" s="2" t="n">
         <v>94.5344963448143</v>
@@ -21955,7 +21965,7 @@
     </row>
     <row r="330">
       <c r="A330" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="B330" s="2" t="n">
         <v>95.3429045631385</v>
@@ -22014,7 +22024,7 @@
     </row>
     <row r="331">
       <c r="A331" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B331" s="2" t="n">
         <v>92.2716309105355</v>
@@ -22073,7 +22083,7 @@
     </row>
     <row r="332">
       <c r="A332" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="B332" s="2" t="n">
         <v>91.1666291091975</v>
@@ -22132,7 +22142,7 @@
     </row>
     <row r="333">
       <c r="A333" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="B333" s="2" t="n">
         <v>90.2360502788793</v>
@@ -22191,7 +22201,7 @@
     </row>
     <row r="334">
       <c r="A334" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="B334" s="2" t="n">
         <v>90.2547058617031</v>
@@ -22250,7 +22260,7 @@
     </row>
     <row r="335">
       <c r="A335" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="B335" s="2" t="n">
         <v>90.5190740970064</v>
@@ -22309,7 +22319,7 @@
     </row>
     <row r="336">
       <c r="A336" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="B336" s="2" t="n">
         <v>89.6221151346543</v>
@@ -22368,7 +22378,7 @@
     </row>
     <row r="337">
       <c r="A337" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="B337" s="2" t="n">
         <v>93.8955237999291</v>
@@ -22427,7 +22437,7 @@
     </row>
     <row r="338">
       <c r="A338" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="B338" s="2" t="n">
         <v>96.4783071320962</v>
@@ -22486,7 +22496,7 @@
     </row>
     <row r="339">
       <c r="A339" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="B339" s="2" t="n">
         <v>97.6434182994192</v>
@@ -22545,7 +22555,7 @@
     </row>
     <row r="340">
       <c r="A340" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="B340" s="2" t="n">
         <v>85.9152891461596</v>
@@ -22604,7 +22614,7 @@
     </row>
     <row r="341">
       <c r="A341" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="B341" s="2" t="n">
         <v>79.1618082991664</v>
@@ -22663,7 +22673,7 @@
     </row>
     <row r="342">
       <c r="A342" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="B342" s="2" t="n">
         <v>48.2692837191472</v>
@@ -22722,7 +22732,7 @@
     </row>
     <row r="343">
       <c r="A343" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="B343" s="2" t="n">
         <v>56.3647415226736</v>
@@ -22781,7 +22791,7 @@
     </row>
     <row r="344">
       <c r="A344" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="B344" s="2" t="n">
         <v>77.13148971026</v>
@@ -22840,7 +22850,7 @@
     </row>
     <row r="345">
       <c r="A345" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="B345" s="2" t="n">
         <v>103.100116789423</v>
@@ -22899,7 +22909,7 @@
     </row>
     <row r="346">
       <c r="A346" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="B346" s="2" t="n">
         <v>106.849741066772</v>
@@ -22958,7 +22968,7 @@
     </row>
     <row r="347">
       <c r="A347" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="B347" s="2" t="n">
         <v>109.158164164525</v>
@@ -23017,7 +23027,7 @@
     </row>
     <row r="348">
       <c r="A348" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="B348" s="2" t="n">
         <v>109.461161541418</v>
@@ -23076,7 +23086,7 @@
     </row>
     <row r="349">
       <c r="A349" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="B349" s="2" t="n">
         <v>107.630905453914</v>
@@ -23135,7 +23145,7 @@
     </row>
     <row r="350">
       <c r="A350" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="B350" s="2" t="n">
         <v>108.341056358602</v>
@@ -23194,7 +23204,7 @@
     </row>
     <row r="351">
       <c r="A351" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="B351" s="2" t="n">
         <v>107.635992948868</v>
@@ -23253,7 +23263,7 @@
     </row>
     <row r="352">
       <c r="A352" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B352" s="2" t="n">
         <v>108.278995218018</v>
@@ -23312,7 +23322,7 @@
     </row>
     <row r="353">
       <c r="A353" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="B353" s="2" t="n">
         <v>118.09812507719</v>
@@ -23371,7 +23381,7 @@
     </row>
     <row r="354">
       <c r="A354" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="B354" s="2" t="n">
         <v>133.344604208749</v>
@@ -23430,7 +23440,7 @@
     </row>
     <row r="355">
       <c r="A355" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B355" s="2" t="n">
         <v>128.116907966277</v>
@@ -23489,7 +23499,7 @@
     </row>
     <row r="356">
       <c r="A356" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="B356" s="2" t="n">
         <v>122.87262192529</v>
@@ -23548,7 +23558,7 @@
     </row>
     <row r="357">
       <c r="A357" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B357" s="2" t="n">
         <v>117.542214855323</v>
@@ -23607,7 +23617,7 @@
     </row>
     <row r="358">
       <c r="A358" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="B358" s="2" t="n">
         <v>113.055028623262</v>
@@ -23666,7 +23676,7 @@
     </row>
     <row r="359">
       <c r="A359" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="B359" s="2" t="n">
         <v>107.04710250073</v>
@@ -23725,7 +23735,7 @@
     </row>
     <row r="360">
       <c r="A360" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="B360" s="2" t="n">
         <v>106.179823532816</v>
@@ -23784,7 +23794,7 @@
     </row>
     <row r="361">
       <c r="A361" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B361" s="2" t="n">
         <v>108.211905880501</v>
@@ -23843,7 +23853,7 @@
     </row>
     <row r="362">
       <c r="A362" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="B362" s="2" t="n">
         <v>106.567599883258</v>
@@ -23902,7 +23912,7 @@
     </row>
     <row r="363">
       <c r="A363" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B363" s="2" t="n">
         <v>105.680719542817</v>
@@ -23961,7 +23971,7 @@
     </row>
     <row r="364">
       <c r="A364" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B364" s="2" t="n">
         <v>102.321024702442</v>
@@ -24020,7 +24030,7 @@
     </row>
     <row r="365">
       <c r="A365" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="B365" s="2" t="n">
         <v>98.6646169448848</v>
@@ -24079,7 +24089,7 @@
     </row>
     <row r="366">
       <c r="A366" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="B366" s="2" t="n">
         <v>95.148900131875</v>
@@ -24138,7 +24148,7 @@
     </row>
     <row r="367">
       <c r="A367" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="B367" s="2" t="n">
         <v>97.0200997383998</v>
@@ -24197,7 +24207,7 @@
     </row>
     <row r="368">
       <c r="A368" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="B368" s="2" t="n">
         <v>92.4245727026426</v>
@@ -24256,7 +24266,7 @@
     </row>
     <row r="369">
       <c r="A369" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="B369" s="2" t="n">
         <v>88.036444240963</v>
@@ -24315,7 +24325,7 @@
     </row>
     <row r="370">
       <c r="A370" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="B370" s="2" t="n">
         <v>89.7982198058401</v>
@@ -24374,7 +24384,7 @@
     </row>
     <row r="371">
       <c r="A371" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="B371" s="2" t="n">
         <v>91.2010024931113</v>
@@ -24433,7 +24443,7 @@
     </row>
     <row r="372">
       <c r="A372" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="B372" s="2" t="n">
         <v>91.6921022435247</v>
@@ -24492,7 +24502,7 @@
     </row>
     <row r="373">
       <c r="A373" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B373" s="2" t="n">
         <v>88.7169590908352</v>
@@ -24551,7 +24561,7 @@
     </row>
     <row r="374">
       <c r="A374" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="B374" s="2" t="n">
         <v>88.2527838806425</v>
@@ -24610,7 +24620,7 @@
     </row>
     <row r="375">
       <c r="A375" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="B375" s="2" t="n">
         <v>90.1138556964084</v>
@@ -24669,7 +24679,7 @@
     </row>
     <row r="376">
       <c r="A376" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="B376" s="2" t="n">
         <v>93.9652266513381</v>
@@ -24728,7 +24738,7 @@
     </row>
     <row r="377">
       <c r="A377" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="B377" s="2" t="n">
         <v>92.8765023738037</v>
@@ -24787,7 +24797,7 @@
     </row>
     <row r="378">
       <c r="A378" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="B378" s="2" t="n">
         <v>95.1692781226711</v>
@@ -24846,7 +24856,7 @@
     </row>
     <row r="379">
       <c r="A379" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="B379" s="2" t="n">
         <v>94.6558123795631</v>
@@ -24905,7 +24915,7 @@
     </row>
     <row r="380">
       <c r="A380" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="B380" s="2" t="n">
         <v>95.5474612238855</v>
@@ -24964,7 +24974,7 @@
     </row>
     <row r="381">
       <c r="A381" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="B381" s="2" t="n">
         <v>93.2392715370596</v>
@@ -25023,7 +25033,7 @@
     </row>
     <row r="382">
       <c r="A382" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="B382" s="2" t="n">
         <v>93.5084342172785</v>
@@ -25082,7 +25092,7 @@
     </row>
     <row r="383">
       <c r="A383" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="B383" s="2" t="n">
         <v>93.469555303468</v>
@@ -25141,7 +25151,7 @@
     </row>
     <row r="384">
       <c r="A384" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="B384" s="2" t="n">
         <v>93.4707191842858</v>
@@ -25200,7 +25210,7 @@
     </row>
     <row r="385">
       <c r="A385" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="B385" s="2" t="n">
         <v>93.7025187315925</v>
@@ -25259,7 +25269,7 @@
     </row>
     <row r="386">
       <c r="A386" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="B386" s="2" t="n">
         <v>94.8069436002527</v>
@@ -25318,7 +25328,7 @@
     </row>
     <row r="387">
       <c r="A387" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="B387" s="2" t="n">
         <v>96.1185079094449</v>
@@ -25377,7 +25387,7 @@
     </row>
     <row r="388">
       <c r="A388" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="B388" s="2" t="n">
         <v>97.2803682877161</v>
@@ -25436,7 +25446,7 @@
     </row>
     <row r="389">
       <c r="A389" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="B389" s="2" t="n">
         <v>98.3194519836946</v>
@@ -25495,7 +25505,7 @@
     </row>
     <row r="390">
       <c r="A390" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="B390" s="2" t="n">
         <v>97.4720932071772</v>
@@ -25554,7 +25564,7 @@
     </row>
     <row r="391">
       <c r="A391" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="B391" s="2" t="n">
         <v>97.4394001650266</v>
@@ -25613,7 +25623,7 @@
     </row>
     <row r="392">
       <c r="A392" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="B392" s="2" t="n">
         <v>97.6664137785381</v>
@@ -25672,7 +25682,7 @@
     </row>
     <row r="393">
       <c r="A393" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="B393" s="2" t="n">
         <v>97.2421035150727</v>
@@ -25731,7 +25741,7 @@
     </row>
     <row r="394">
       <c r="A394" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="B394" s="2" t="n">
         <v>97.4012611817873</v>
@@ -25790,7 +25800,7 @@
     </row>
     <row r="395">
       <c r="A395" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="B395" s="2" t="n">
         <v>97.9695612904388</v>
@@ -25849,7 +25859,7 @@
     </row>
     <row r="396">
       <c r="A396" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="B396" s="2" t="n">
         <v>100.574626793105</v>
@@ -25908,7 +25918,7 @@
     </row>
     <row r="397">
       <c r="A397" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="B397" s="2" t="n">
         <v>101.474423021452</v>
@@ -25967,7 +25977,7 @@
     </row>
     <row r="398">
       <c r="A398" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="B398" s="2" t="n">
         <v>101.107471966189</v>
@@ -26026,7 +26036,7 @@
     </row>
     <row r="399">
       <c r="A399" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="B399" s="2" t="n">
         <v>100.742379185402</v>
@@ -26085,7 +26095,7 @@
     </row>
     <row r="400">
       <c r="A400" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="B400" s="2" t="n">
         <v>100.715685524868</v>
@@ -26144,7 +26154,7 @@
     </row>
     <row r="401">
       <c r="A401" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="B401" s="2" t="n">
         <v>98.8583844520579</v>
@@ -26203,7 +26213,7 @@
     </row>
     <row r="402">
       <c r="A402" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="B402" s="2" t="n">
         <v>94.1097217292409</v>
@@ -26262,7 +26272,7 @@
     </row>
     <row r="403">
       <c r="A403" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="B403" s="2" t="n">
         <v>96.1610373935028</v>
@@ -26321,7 +26331,7 @@
     </row>
     <row r="404">
       <c r="A404" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="B404" s="2" t="n">
         <v>97.7375885526721</v>
@@ -26380,7 +26390,7 @@
     </row>
     <row r="405">
       <c r="A405" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="B405" s="2" t="n">
         <v>100.280466282684</v>
@@ -26439,7 +26449,7 @@
     </row>
     <row r="406">
       <c r="A406" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="B406" s="2" t="n">
         <v>101.231111652883</v>
@@ -26498,7 +26508,7 @@
     </row>
     <row r="407">
       <c r="A407" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="B407" s="2" t="n">
         <v>100.921315733302</v>
@@ -26557,7 +26567,7 @@
     </row>
     <row r="408">
       <c r="A408" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="B408" s="2" t="n">
         <v>98.7699004474908</v>
@@ -26616,7 +26626,7 @@
     </row>
     <row r="409">
       <c r="A409" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="B409" s="2" t="n">
         <v>100.221855743791</v>
@@ -26675,7 +26685,7 @@
     </row>
     <row r="410">
       <c r="A410" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="B410" s="2" t="n">
         <v>100.676245904946</v>
@@ -26734,7 +26744,7 @@
     </row>
     <row r="411">
       <c r="A411" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="B411" s="2" t="n">
         <v>101.079892423582</v>
@@ -26793,7 +26803,7 @@
     </row>
     <row r="412">
       <c r="A412" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="B412" s="2" t="n">
         <v>100.364770088857</v>
@@ -26852,7 +26862,7 @@
     </row>
     <row r="413">
       <c r="A413" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="B413" s="2" t="n">
         <v>102.22117234763</v>
@@ -26911,7 +26921,7 @@
     </row>
     <row r="414">
       <c r="A414" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="B414" s="2" t="n">
         <v>100.294367560849</v>
@@ -26970,7 +26980,7 @@
     </row>
     <row r="415">
       <c r="A415" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="B415" s="2" t="n">
         <v>101.155674803057</v>
@@ -27029,7 +27039,7 @@
     </row>
     <row r="416">
       <c r="A416" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="B416" s="2"/>
       <c r="C416" s="3" t="n">
@@ -27062,7 +27072,7 @@
     </row>
     <row r="417">
       <c r="A417" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="B417" s="2"/>
       <c r="C417" s="3" t="n">
@@ -27095,7 +27105,7 @@
     </row>
     <row r="418">
       <c r="A418" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="B418" s="2"/>
       <c r="C418" s="3" t="n">
@@ -27128,7 +27138,7 @@
     </row>
     <row r="419">
       <c r="A419" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="B419" s="2"/>
       <c r="C419" s="3" t="n">
@@ -27161,7 +27171,7 @@
     </row>
     <row r="420">
       <c r="A420" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="B420" s="2"/>
       <c r="C420" s="3" t="n">
@@ -27194,7 +27204,7 @@
     </row>
     <row r="421">
       <c r="A421" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="B421" s="2"/>
       <c r="C421" s="3" t="n">
@@ -27227,7 +27237,7 @@
     </row>
     <row r="422">
       <c r="A422" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="B422" s="2"/>
       <c r="C422" s="3" t="n">
@@ -27260,7 +27270,7 @@
     </row>
     <row r="423">
       <c r="A423" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="B423" s="2"/>
       <c r="C423" s="3" t="n">
@@ -27293,7 +27303,7 @@
     </row>
     <row r="424">
       <c r="A424" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="B424" s="2"/>
       <c r="C424" s="3" t="n">
@@ -27326,7 +27336,7 @@
     </row>
     <row r="425">
       <c r="A425" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B425" s="2"/>
       <c r="C425" s="3" t="n">
@@ -27359,7 +27369,7 @@
     </row>
     <row r="426">
       <c r="A426" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="B426" s="2"/>
       <c r="C426" s="3" t="n">
@@ -27392,7 +27402,7 @@
     </row>
     <row r="427">
       <c r="A427" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="B427" s="2"/>
       <c r="C427" s="3" t="n">
@@ -27425,7 +27435,7 @@
     </row>
     <row r="428">
       <c r="A428" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="B428" s="2"/>
       <c r="C428" s="3"/>
@@ -27448,7 +27458,7 @@
     </row>
     <row r="429">
       <c r="A429" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="B429" s="2"/>
       <c r="C429" s="3"/>
@@ -27471,7 +27481,7 @@
     </row>
     <row r="430">
       <c r="A430" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="B430" s="2"/>
       <c r="C430" s="3"/>
@@ -27494,7 +27504,7 @@
     </row>
     <row r="431">
       <c r="A431" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="B431" s="2"/>
       <c r="C431" s="3"/>
@@ -27517,7 +27527,7 @@
     </row>
     <row r="432">
       <c r="A432" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="B432" s="2"/>
       <c r="C432" s="3"/>
@@ -27540,7 +27550,7 @@
     </row>
     <row r="433">
       <c r="A433" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="B433" s="2"/>
       <c r="C433" s="3"/>
@@ -27563,7 +27573,7 @@
     </row>
     <row r="434">
       <c r="A434" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="B434" s="2"/>
       <c r="C434" s="3"/>
@@ -27586,7 +27596,7 @@
     </row>
     <row r="435">
       <c r="A435" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="B435" s="2"/>
       <c r="C435" s="3"/>
@@ -27609,7 +27619,7 @@
     </row>
     <row r="436">
       <c r="A436" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="B436" s="2"/>
       <c r="C436" s="3"/>
@@ -27632,7 +27642,7 @@
     </row>
     <row r="437">
       <c r="A437" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="B437" s="2"/>
       <c r="C437" s="3"/>
@@ -27655,7 +27665,7 @@
     </row>
     <row r="438">
       <c r="A438" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="B438" s="2"/>
       <c r="C438" s="3"/>
@@ -27678,7 +27688,7 @@
     </row>
     <row r="439">
       <c r="A439" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="B439" s="2"/>
       <c r="C439" s="3"/>
@@ -27701,7 +27711,7 @@
     </row>
     <row r="440">
       <c r="A440" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="B440" s="2"/>
       <c r="C440" s="3"/>
@@ -27724,7 +27734,7 @@
     </row>
     <row r="441">
       <c r="A441" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="B441" s="2"/>
       <c r="C441" s="3"/>
@@ -27747,7 +27757,7 @@
     </row>
     <row r="442">
       <c r="A442" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="B442" s="2"/>
       <c r="C442" s="3"/>
@@ -27770,7 +27780,7 @@
     </row>
     <row r="443">
       <c r="A443" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="B443" s="2"/>
       <c r="C443" s="3"/>
@@ -27793,7 +27803,7 @@
     </row>
     <row r="444">
       <c r="A444" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="B444" s="2"/>
       <c r="C444" s="3"/>
@@ -27816,7 +27826,7 @@
     </row>
     <row r="445">
       <c r="A445" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="B445" s="2"/>
       <c r="C445" s="3"/>
@@ -27839,7 +27849,7 @@
     </row>
     <row r="446">
       <c r="A446" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="B446" s="2"/>
       <c r="C446" s="3"/>
@@ -27862,7 +27872,7 @@
     </row>
     <row r="447">
       <c r="A447" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="B447" s="2"/>
       <c r="C447" s="3"/>
@@ -27885,7 +27895,7 @@
     </row>
     <row r="448">
       <c r="A448" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="B448" s="2"/>
       <c r="C448" s="3"/>
@@ -27908,7 +27918,7 @@
     </row>
     <row r="449">
       <c r="A449" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="B449" s="2"/>
       <c r="C449" s="3"/>
@@ -27931,7 +27941,7 @@
     </row>
     <row r="450">
       <c r="A450" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="B450" s="2"/>
       <c r="C450" s="3"/>
@@ -27954,7 +27964,7 @@
     </row>
     <row r="451">
       <c r="A451" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="B451" s="2"/>
       <c r="C451" s="3"/>
@@ -27977,7 +27987,7 @@
     </row>
     <row r="452">
       <c r="A452" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="B452" s="2"/>
       <c r="C452" s="3"/>
@@ -28000,7 +28010,7 @@
     </row>
     <row r="453">
       <c r="A453" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="B453" s="2"/>
       <c r="C453" s="3"/>
@@ -28023,7 +28033,7 @@
     </row>
     <row r="454">
       <c r="A454" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="B454" s="2"/>
       <c r="C454" s="3"/>
@@ -28046,7 +28056,7 @@
     </row>
     <row r="455">
       <c r="A455" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="B455" s="2"/>
       <c r="C455" s="3"/>
@@ -28069,7 +28079,7 @@
     </row>
     <row r="456">
       <c r="A456" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="B456" s="2"/>
       <c r="C456" s="3"/>
@@ -28092,7 +28102,7 @@
     </row>
     <row r="457">
       <c r="A457" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="B457" s="2"/>
       <c r="C457" s="3"/>
@@ -28115,7 +28125,7 @@
     </row>
     <row r="458">
       <c r="A458" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="B458" s="2"/>
       <c r="C458" s="3"/>
@@ -28138,7 +28148,7 @@
     </row>
     <row r="459">
       <c r="A459" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="B459" s="2"/>
       <c r="C459" s="3"/>
@@ -28161,7 +28171,7 @@
     </row>
     <row r="460">
       <c r="A460" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="B460" s="2"/>
       <c r="C460" s="3"/>
@@ -28184,7 +28194,7 @@
     </row>
     <row r="461">
       <c r="A461" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="B461" s="2"/>
       <c r="C461" s="3"/>
@@ -28207,7 +28217,7 @@
     </row>
     <row r="462">
       <c r="A462" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="B462" s="2"/>
       <c r="C462" s="3"/>
@@ -28230,7 +28240,7 @@
     </row>
     <row r="463">
       <c r="A463" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="B463" s="2"/>
       <c r="C463" s="3"/>
@@ -28253,7 +28263,7 @@
     </row>
     <row r="464">
       <c r="A464" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="B464" s="2"/>
       <c r="C464" s="3"/>
@@ -28276,7 +28286,7 @@
     </row>
     <row r="465">
       <c r="A465" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="B465" s="2"/>
       <c r="C465" s="3"/>
@@ -28299,7 +28309,7 @@
     </row>
     <row r="466">
       <c r="A466" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="B466" s="2"/>
       <c r="C466" s="3"/>
@@ -28322,7 +28332,7 @@
     </row>
     <row r="467">
       <c r="A467" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="B467" s="2"/>
       <c r="C467" s="3"/>
@@ -28345,7 +28355,7 @@
     </row>
     <row r="468">
       <c r="A468" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="B468" s="2"/>
       <c r="C468" s="3"/>
@@ -28368,7 +28378,7 @@
     </row>
     <row r="469">
       <c r="A469" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="B469" s="2"/>
       <c r="C469" s="3"/>
@@ -28402,97 +28412,97 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
     </row>
   </sheetData>
@@ -28516,7 +28526,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="B2" s="1"/>
     </row>
@@ -28526,13 +28536,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>0.154914895533662</v>
@@ -28540,7 +28550,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>0.160690921916846</v>
@@ -28548,7 +28558,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>0.152518003044176</v>
@@ -28556,7 +28566,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>0.127681676842972</v>
@@ -28564,7 +28574,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>0.0864746883894524</v>
@@ -28572,7 +28582,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>0.0535581973596299</v>
@@ -28580,7 +28590,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>0.0573310282123859</v>
@@ -28588,7 +28598,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>0.0959046480080881</v>
@@ -28596,7 +28606,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>0.132677129434212</v>
@@ -28604,7 +28614,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>0.149131690590653</v>
@@ -28612,7 +28622,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>0.138669873804167</v>
@@ -28620,7 +28630,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>0.0870503319994589</v>
@@ -28628,7 +28638,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>-0.00751569471654186</v>
@@ -28636,7 +28646,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>-0.111982764222129</v>
@@ -28644,7 +28654,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>-0.174775157568788</v>
@@ -28652,7 +28662,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>-0.179967759729582</v>
@@ -28660,7 +28670,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>-0.169820453188065</v>
@@ -28668,7 +28678,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>-0.171877807139163</v>
@@ -28676,7 +28686,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>-0.172581230500034</v>

</xml_diff>